<commit_message>
Fix Excel corruption in P13/P1/P2 packs + set P13 to paid (EUR29, §41)
Excel reported 'we found a problem with content'. Two root causes:
- P13 sheet tab name exceeded Excel's 31-char limit (32: '02 · Mock Audit ·
  Skúšobný audit') -> shortened to '… · Skúška'; builder asserts <=31 now
- DEMO builders used insert_rows(), which corrupts merged-cell/CF ranges in
  openpyxl. Replaced in P13, P1 and P2 with a non-destructive 'DEMO Preview ·
  Ukážka' notice sheet + read-only protection.
All 6 product workbooks re-validated: XML well-formed, tabs <=31, zero
merged-range overlaps. (LibreOffice is non-functional in this sandbox, so
validation is openpyxl reload + zip/XML parse + overlap check.)

§41 (Samuel): sell P13 rather than give it away. DB P13 -> EUR29 launch test,
tier 'pack' (was EUR0/free); seed_compliance updated + re-seeded; validate.py
green (24 products, 0 free-tier). README + handover updated.

https://claude.ai/code/session_01KgoUQQxKev7bA6vz6wTYg2
</commit_message>
<xml_diff>
--- a/asset-forge/products/P13_Compliance_Gap_Analysis_Mock_Audit.xlsx
+++ b/asset-forge/products/P13_Compliance_Gap_Analysis_Mock_Audit.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="00 · Start Here · Začnite tu" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="01 · Gap Analysis · Analýza" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02 · Mock Audit · Skúšobný audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="02 · Mock Audit · Skúška" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03 · Readiness · Pripravenosť" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="04 · Next Steps · Ďalšie kroky" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -1063,7 +1063,7 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>ASSET-FORGE · v1.0 · 30/05/2026 · EU (Ireland) · FREE lead magnet · Template only — not legal advice nor a guarantee of certification. · Šablóna — nie je právne poradenstvo ani záruka certifikácie.</t>
+          <t>ASSET-FORGE · v1.1 · 30/05/2026 · EU (Ireland) · FREE lead magnet · Template only — not legal advice nor a guarantee of certification. · Šablóna — nie je právne poradenstvo ani záruka certifikácie.</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
       <c r="B5" s="27" t="n"/>
       <c r="C5" s="28" t="n"/>
       <c r="D5" s="29">
-        <f>IF('02 · Mock Audit · Skúšobný audit'!D28="","",'02 · Mock Audit · Skúšobný audit'!D28)</f>
+        <f>IF('02 · Mock Audit · Skúška'!D28="","",'02 · Mock Audit · Skúška'!D28)</f>
         <v/>
       </c>
       <c r="E5" s="27" t="n"/>
@@ -2569,7 +2569,7 @@
       <c r="B6" s="27" t="n"/>
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="30">
-        <f>IF(AND('01 · Gap Analysis · Analýza'!E35="",'02 · Mock Audit · Skúšobný audit'!D28=""),"",IF('01 · Gap Analysis · Analýza'!E35="",'02 · Mock Audit · Skúšobný audit'!D28,IF('02 · Mock Audit · Skúšobný audit'!D28="",'01 · Gap Analysis · Analýza'!E35,('01 · Gap Analysis · Analýza'!E35+'02 · Mock Audit · Skúšobný audit'!D28)/2)))</f>
+        <f>IF(AND('01 · Gap Analysis · Analýza'!E35="",'02 · Mock Audit · Skúška'!D28=""),"",IF('01 · Gap Analysis · Analýza'!E35="",'02 · Mock Audit · Skúška'!D28,IF('02 · Mock Audit · Skúška'!D28="",'01 · Gap Analysis · Analýza'!E35,('01 · Gap Analysis · Analýza'!E35+'02 · Mock Audit · Skúška'!D28)/2)))</f>
         <v/>
       </c>
       <c r="E6" s="27" t="n"/>

</xml_diff>